<commit_message>
Finalize GreenLeaf Task 2 control mapping and README
</commit_message>
<xml_diff>
--- a/Control_Mapping.xlsx
+++ b/Control_Mapping.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="402">
   <si>
     <t xml:space="preserve">Control ID</t>
   </si>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">Organizational</t>
   </si>
   <si>
-    <t xml:space="preserve">Not Assessed</t>
+    <t xml:space="preserve">Partial</t>
   </si>
   <si>
     <t xml:space="preserve">Information Security Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Information Security Policy reference template found; no GreenLeaf approval, publication, or periodic review evidence.</t>
+    <t xml:space="preserve">Information Security Policy reference template found; no GreenLeaf approval, publication, or periodic review evidence. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Approve an organization-specific policy, assign an owner, communicate it, and establish a review cycle.</t>
@@ -71,10 +71,13 @@
     <t xml:space="preserve">Information security roles and responsibilities</t>
   </si>
   <si>
+    <t xml:space="preserve">Not Implemented</t>
+  </si>
+  <si>
     <t xml:space="preserve">Missing (no reference template mapped)</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security roles and responsibilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security roles and responsibilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security roles and responsibilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -86,7 +89,7 @@
     <t xml:space="preserve">Segregation of duties</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for segregation of duties; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for segregation of duties; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of segregation of duties, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -98,7 +101,7 @@
     <t xml:space="preserve">Management responsibilities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for management responsibilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for management responsibilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of management responsibilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -110,7 +113,7 @@
     <t xml:space="preserve">Contact with authorities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for contact with authorities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for contact with authorities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of contact with authorities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -122,7 +125,7 @@
     <t xml:space="preserve">Contact with special interest groups</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for contact with special interest groups; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for contact with special interest groups; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of contact with special interest groups, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -134,7 +137,7 @@
     <t xml:space="preserve">Threat intelligence</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for threat intelligence; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for threat intelligence; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of threat intelligence, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -146,7 +149,7 @@
     <t xml:space="preserve">Information security in project management</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security in project management; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security in project management; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security in project management, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -158,7 +161,7 @@
     <t xml:space="preserve">Inventory of information and other associated assets</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for inventory of information and other associated assets; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for inventory of information and other associated assets; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of inventory of information and other associated assets, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -170,7 +173,7 @@
     <t xml:space="preserve">Acceptable use of information and other associated assets</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for acceptable use of information and other associated assets; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for acceptable use of information and other associated assets; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of acceptable use of information and other associated assets, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -182,7 +185,7 @@
     <t xml:space="preserve">Return of assets</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for return of assets; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for return of assets; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of return of assets, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -197,7 +200,7 @@
     <t xml:space="preserve">Data Classification Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Data classification template found; no approved GreenLeaf classification scheme evidenced. Demo records are fictional.</t>
+    <t xml:space="preserve">Data classification template found; no approved GreenLeaf classification scheme evidenced. Demo records are fictional. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Define classification levels and handling rules for real borrower and financial data.</t>
@@ -209,7 +212,7 @@
     <t xml:space="preserve">Labelling of information</t>
   </si>
   <si>
-    <t xml:space="preserve">Data classification template found; no evidence of GreenLeaf labelling practices.</t>
+    <t xml:space="preserve">Data classification template found; no evidence of GreenLeaf labelling practices. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Define labels and verify labels on representative information assets.</t>
@@ -221,7 +224,7 @@
     <t xml:space="preserve">Information transfer</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information transfer; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information transfer; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information transfer, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -236,7 +239,7 @@
     <t xml:space="preserve">Access Control Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">External access-control template identified, but not adopted by fictional GreenLeaf; public demo borrower route has no access restriction.</t>
+    <t xml:space="preserve">External access-control template identified, but not adopted by fictional GreenLeaf; public demo borrower route has no access restriction. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Approve a GreenLeaf-specific access-control policy, define roles and access reviews, and enforce authorization on protected routes.</t>
@@ -248,7 +251,7 @@
     <t xml:space="preserve">Identity management</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for identity management; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for identity management; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of identity management, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -260,7 +263,7 @@
     <t xml:space="preserve">Authentication information</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for authentication information; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for authentication information; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of authentication information, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -272,7 +275,7 @@
     <t xml:space="preserve">Access rights</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for access rights; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for access rights; applicability and operating effectiveness not assessed. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of access rights, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -284,7 +287,7 @@
     <t xml:space="preserve">Information security in supplier relationships</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security in supplier relationships; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security in supplier relationships; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security in supplier relationships, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -296,7 +299,7 @@
     <t xml:space="preserve">Addressing information security within supplier agreements</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for addressing information security within supplier agreements; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for addressing information security within supplier agreements; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of addressing information security within supplier agreements, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -308,7 +311,7 @@
     <t xml:space="preserve">Managing information security in the ICT supply chain</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for managing information security in the ict supply chain; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for managing information security in the ict supply chain; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of managing information security in the ict supply chain, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -320,7 +323,7 @@
     <t xml:space="preserve">Monitoring, review and change management of supplier services</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for monitoring, review and change management of supplier services; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for monitoring, review and change management of supplier services; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of monitoring, review and change management of supplier services, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -332,7 +335,7 @@
     <t xml:space="preserve">Information security for use of cloud services</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security for use of cloud services; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security for use of cloud services; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security for use of cloud services, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -347,7 +350,7 @@
     <t xml:space="preserve">Incident Response Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Incident-response reference template found; no GreenLeaf incident plan approval or exercises evidenced.</t>
+    <t xml:space="preserve">Incident-response reference template found; no GreenLeaf incident plan approval or exercises evidenced. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Approve an incident management plan with responsibilities, escalation, and testing.</t>
@@ -359,7 +362,7 @@
     <t xml:space="preserve">Assessment and decision on information security events</t>
   </si>
   <si>
-    <t xml:space="preserve">Incident-response template found; no evidence of triage or severity decision workflow.</t>
+    <t xml:space="preserve">Incident-response template found; no evidence of triage or severity decision workflow. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Define event assessment criteria and retain triage decision records.</t>
@@ -371,7 +374,7 @@
     <t xml:space="preserve">Response to information security incidents</t>
   </si>
   <si>
-    <t xml:space="preserve">Incident-response template found; no evidence of exercised response procedures.</t>
+    <t xml:space="preserve">Incident-response template found; no evidence of exercised response procedures. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Define response playbooks and conduct a tabletop exercise.</t>
@@ -383,7 +386,7 @@
     <t xml:space="preserve">Learning from information security incidents</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for learning from information security incidents; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for learning from information security incidents; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of learning from information security incidents, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -395,7 +398,7 @@
     <t xml:space="preserve">Collection of evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for collection of evidence; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for collection of evidence; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of collection of evidence, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -410,7 +413,7 @@
     <t xml:space="preserve">Business Continuity Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Business continuity template found; no GreenLeaf continuity plan or exercise evidence.</t>
+    <t xml:space="preserve">Business continuity template found; no GreenLeaf continuity plan or exercise evidence. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Document information security requirements during disruptions and test continuity arrangements.</t>
@@ -422,7 +425,7 @@
     <t xml:space="preserve">ICT readiness for business continuity</t>
   </si>
   <si>
-    <t xml:space="preserve">Business continuity template found; no recovery objectives or ICT recovery test evidenced.</t>
+    <t xml:space="preserve">Business continuity template found; no recovery objectives or ICT recovery test evidenced. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Define recovery targets and conduct an ICT recovery test.</t>
@@ -434,7 +437,7 @@
     <t xml:space="preserve">Legal, statutory, regulatory and contractual requirements</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for legal, statutory, regulatory and contractual requirements; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for legal, statutory, regulatory and contractual requirements; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of legal, statutory, regulatory and contractual requirements, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -446,7 +449,7 @@
     <t xml:space="preserve">Intellectual property rights</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for intellectual property rights; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for intellectual property rights; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of intellectual property rights, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -458,7 +461,7 @@
     <t xml:space="preserve">Protection of records</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection of records; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection of records; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of protection of records, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -470,7 +473,7 @@
     <t xml:space="preserve">Privacy and protection of PII</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for privacy and protection of pii; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for privacy and protection of pii; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of privacy and protection of pii, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -482,7 +485,7 @@
     <t xml:space="preserve">Independent review of information security</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for independent review of information security; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for independent review of information security; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of independent review of information security, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -494,7 +497,7 @@
     <t xml:space="preserve">Compliance with policies, rules and standards for information security</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for compliance with policies, rules and standards for information security; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for compliance with policies, rules and standards for information security; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of compliance with policies, rules and standards for information security, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -506,7 +509,7 @@
     <t xml:space="preserve">Documented operating procedures</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for documented operating procedures; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for documented operating procedures; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of documented operating procedures, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -521,7 +524,7 @@
     <t xml:space="preserve">People</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for screening; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for screening; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of screening, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -533,7 +536,7 @@
     <t xml:space="preserve">Terms and conditions of employment</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for terms and conditions of employment; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for terms and conditions of employment; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of terms and conditions of employment, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -545,7 +548,7 @@
     <t xml:space="preserve">Information security awareness, education and training</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security awareness, education and training; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security awareness, education and training; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security awareness, education and training, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -557,7 +560,7 @@
     <t xml:space="preserve">Disciplinary process</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for disciplinary process; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for disciplinary process; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of disciplinary process, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -569,7 +572,7 @@
     <t xml:space="preserve">Responsibilities after termination or change of employment</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for responsibilities after termination or change of employment; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for responsibilities after termination or change of employment; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of responsibilities after termination or change of employment, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -581,7 +584,7 @@
     <t xml:space="preserve">Confidentiality or non-disclosure agreements</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for confidentiality or non-disclosure agreements; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for confidentiality or non-disclosure agreements; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of confidentiality or non-disclosure agreements, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -593,7 +596,7 @@
     <t xml:space="preserve">Remote working</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for remote working; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for remote working; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of remote working, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -605,7 +608,7 @@
     <t xml:space="preserve">Information security event reporting</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security event reporting; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information security event reporting; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information security event reporting, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -620,7 +623,7 @@
     <t xml:space="preserve">Physical</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical security perimeters; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical security perimeters; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of physical security perimeters, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -632,7 +635,7 @@
     <t xml:space="preserve">Physical entry</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical entry; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical entry; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of physical entry, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -644,7 +647,7 @@
     <t xml:space="preserve">Securing offices, rooms and facilities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for securing offices, rooms and facilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for securing offices, rooms and facilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of securing offices, rooms and facilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -656,7 +659,7 @@
     <t xml:space="preserve">Physical security monitoring</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical security monitoring; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for physical security monitoring; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of physical security monitoring, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -668,7 +671,7 @@
     <t xml:space="preserve">Protecting against physical and environmental threats</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protecting against physical and environmental threats; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protecting against physical and environmental threats; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of protecting against physical and environmental threats, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -680,7 +683,7 @@
     <t xml:space="preserve">Working in secure areas</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for working in secure areas; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for working in secure areas; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of working in secure areas, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -692,7 +695,7 @@
     <t xml:space="preserve">Clear desk and clear screen</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for clear desk and clear screen; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for clear desk and clear screen; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of clear desk and clear screen, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -704,7 +707,7 @@
     <t xml:space="preserve">Equipment siting and protection</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for equipment siting and protection; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for equipment siting and protection; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of equipment siting and protection, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -716,7 +719,7 @@
     <t xml:space="preserve">Security of assets off-premises</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security of assets off-premises; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security of assets off-premises; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of security of assets off-premises, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -728,7 +731,7 @@
     <t xml:space="preserve">Storage media</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for storage media; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for storage media; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of storage media, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -740,7 +743,7 @@
     <t xml:space="preserve">Supporting utilities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for supporting utilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for supporting utilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of supporting utilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -752,7 +755,7 @@
     <t xml:space="preserve">Cabling security</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for cabling security; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for cabling security; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of cabling security, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -764,7 +767,7 @@
     <t xml:space="preserve">Equipment maintenance</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for equipment maintenance; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for equipment maintenance; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of equipment maintenance, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -776,7 +779,7 @@
     <t xml:space="preserve">Secure disposal or re-use of equipment</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure disposal or re-use of equipment; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure disposal or re-use of equipment; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of secure disposal or re-use of equipment, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -791,7 +794,7 @@
     <t xml:space="preserve">Technological</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for user endpoint devices; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for user endpoint devices; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of user endpoint devices, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -803,7 +806,7 @@
     <t xml:space="preserve">Privileged access rights</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for privileged access rights; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for privileged access rights; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of privileged access rights, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -815,7 +818,7 @@
     <t xml:space="preserve">Information access restriction</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandbox /borrowers returns fictional records without authentication; behavior observed on the public demonstration. This does not establish real borrower-data exposure.</t>
+    <t xml:space="preserve">Sandbox /borrowers returns fictional records without authentication; behavior observed on the public demonstration. This does not establish real borrower-data exposure. Simulated rating is limited to the demonstration borrower endpoint.</t>
   </si>
   <si>
     <t xml:space="preserve">Require server-side authentication and role-based authorization before any real borrower records are accessible; verify denial of anonymous requests.</t>
@@ -827,7 +830,7 @@
     <t xml:space="preserve">Access to source code</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for access to source code; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for access to source code; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of access to source code, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -839,7 +842,7 @@
     <t xml:space="preserve">Secure authentication</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandbox /login is explicitly demonstration-only with a disabled button; source code has no login/session handler.</t>
+    <t xml:space="preserve">Sandbox /login is explicitly demonstration-only with a disabled button; source code has no login/session handler. Simulated rating is limited to the demonstration login flow.</t>
   </si>
   <si>
     <t xml:space="preserve">Implement secure server-side authentication and sessions before any real user or sensitive data is introduced.</t>
@@ -851,7 +854,7 @@
     <t xml:space="preserve">Capacity management</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for capacity management; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for capacity management; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of capacity management, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -863,7 +866,7 @@
     <t xml:space="preserve">Protection against malware</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection against malware; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection against malware; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of protection against malware, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -875,7 +878,7 @@
     <t xml:space="preserve">Management of technical vulnerabilities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for management of technical vulnerabilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for management of technical vulnerabilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of management of technical vulnerabilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -887,7 +890,7 @@
     <t xml:space="preserve">Configuration management</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for configuration management; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for configuration management; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of configuration management, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -899,7 +902,7 @@
     <t xml:space="preserve">Information deletion</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information deletion; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information deletion; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information deletion, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -911,7 +914,7 @@
     <t xml:space="preserve">Data masking</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for data masking; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for data masking; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of data masking, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -923,7 +926,7 @@
     <t xml:space="preserve">Data leakage prevention</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for data leakage prevention; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for data leakage prevention; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of data leakage prevention, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -935,7 +938,7 @@
     <t xml:space="preserve">Information backup</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information backup; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for information backup; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of information backup, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -947,7 +950,7 @@
     <t xml:space="preserve">Redundancy of information processing facilities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for redundancy of information processing facilities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for redundancy of information processing facilities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of redundancy of information processing facilities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -959,7 +962,7 @@
     <t xml:space="preserve">Logging</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for logging; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for logging; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of logging, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -971,7 +974,7 @@
     <t xml:space="preserve">Monitoring activities</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for monitoring activities; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for monitoring activities; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of monitoring activities, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -983,7 +986,7 @@
     <t xml:space="preserve">Clock synchronization</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for clock synchronization; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for clock synchronization; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of clock synchronization, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -995,7 +998,7 @@
     <t xml:space="preserve">Use of privileged utility programs</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for use of privileged utility programs; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for use of privileged utility programs; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of use of privileged utility programs, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1007,7 +1010,7 @@
     <t xml:space="preserve">Installation of software on operational systems</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for installation of software on operational systems; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for installation of software on operational systems; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of installation of software on operational systems, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1019,7 +1022,7 @@
     <t xml:space="preserve">Networks security</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for networks security; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for networks security; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of networks security, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1031,7 +1034,7 @@
     <t xml:space="preserve">Security of network services</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security of network services; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security of network services; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of security of network services, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1043,7 +1046,7 @@
     <t xml:space="preserve">Segregation of networks</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for segregation of networks; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for segregation of networks; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of segregation of networks, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1055,7 +1058,7 @@
     <t xml:space="preserve">Web filtering</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for web filtering; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for web filtering; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of web filtering, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1067,7 +1070,7 @@
     <t xml:space="preserve">Use of cryptography</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for use of cryptography; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for use of cryptography; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of use of cryptography, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1079,7 +1082,7 @@
     <t xml:space="preserve">Secure development life cycle</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure development life cycle; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure development life cycle; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of secure development life cycle, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1091,7 +1094,7 @@
     <t xml:space="preserve">Application security requirements</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for application security requirements; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for application security requirements; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of application security requirements, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1103,7 +1106,7 @@
     <t xml:space="preserve">Secure system architecture and engineering principles</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure system architecture and engineering principles; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure system architecture and engineering principles; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of secure system architecture and engineering principles, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1115,7 +1118,7 @@
     <t xml:space="preserve">Secure coding</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure coding; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for secure coding; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of secure coding, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1127,7 +1130,7 @@
     <t xml:space="preserve">Security testing in development and acceptance</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security testing in development and acceptance; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for security testing in development and acceptance; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of security testing in development and acceptance, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1139,7 +1142,7 @@
     <t xml:space="preserve">Outsourced development</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for outsourced development; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for outsourced development; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of outsourced development, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1151,7 +1154,7 @@
     <t xml:space="preserve">Separation of development, test and production environments</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for separation of development, test and production environments; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for separation of development, test and production environments; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of separation of development, test and production environments, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1166,7 +1169,7 @@
     <t xml:space="preserve">Change Management Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Change-management reference template found; no GreenLeaf approval workflow or change records evidenced.</t>
+    <t xml:space="preserve">Change-management reference template found; no GreenLeaf approval workflow or change records evidenced. Simulated rating: relevant external policy template exists, but organizational adoption and operating effectiveness are not demonstrated.</t>
   </si>
   <si>
     <t xml:space="preserve">Document change approvals, testing, rollback plans, and evidence of completed reviews.</t>
@@ -1178,7 +1181,7 @@
     <t xml:space="preserve">Test information</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for test information; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for test information; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of test information, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1190,7 +1193,7 @@
     <t xml:space="preserve">Protection of information systems during audit testing</t>
   </si>
   <si>
-    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection of information systems during audit testing; applicability and operating effectiveness not assessed.</t>
+    <t xml:space="preserve">No GreenLeaf implementation evidence supplied for protection of information systems during audit testing; applicability and operating effectiveness not assessed. Simulated rating: no mapped policy or demonstrated technical implementation within the supplied assessment evidence; this is not a finding about a real organization.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm applicability of protection of information systems during audit testing, request owner-approved documentation and operational evidence, then assess effectiveness.</t>
@@ -1230,15 +1233,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1254,6 +1261,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1286,7 +1299,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE5E7EB"/>
-        <bgColor rgb="FFFEE2E2"/>
+        <bgColor rgb="FFD8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1299,7 +1312,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1323,72 +1336,80 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="24" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="13">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal" xfId="20"/>
+    <cellStyle name="Comma" xfId="20"/>
+    <cellStyle name="Comma [0]" xfId="21"/>
+    <cellStyle name="Currency" xfId="22"/>
+    <cellStyle name="Currency [0]" xfId="23"/>
+    <cellStyle name="Normal" xfId="24"/>
+    <cellStyle name="Normal 1" xfId="25"/>
+    <cellStyle name="Percent" xfId="26"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDCFCE7"/>
+          <bgColor rgb="FFD8F3DC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFEF3C7"/>
+          <bgColor rgb="FFFFF1B8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE5E7EB"/>
+          <bgColor rgb="FFFADBD8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1413,8 +1434,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFEF3C7"/>
-      <rgbColor rgb="FFDCFCE7"/>
+      <rgbColor rgb="FFFFF1B8"/>
+      <rgbColor rgb="FFE5E7EB"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1428,13 +1449,13 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFE5E7EB"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFD8F3DC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFEE2E2"/>
+      <rgbColor rgb="FFFADBD8"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1698,231 +1719,231 @@
         <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>9</v>
@@ -1931,21 +1952,21 @@
         <v>10</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>9</v>
@@ -1954,44 +1975,44 @@
         <v>10</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>9</v>
@@ -2000,67 +2021,67 @@
         <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>9</v>
@@ -2069,136 +2090,136 @@
         <v>10</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>9</v>
@@ -2207,21 +2228,21 @@
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>9</v>
@@ -2230,21 +2251,21 @@
         <v>10</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>9</v>
@@ -2253,67 +2274,67 @@
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>9</v>
@@ -2322,21 +2343,21 @@
         <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>9</v>
@@ -2345,1462 +2366,1462 @@
         <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="64" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -3814,13 +3835,10 @@
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>D2="Not Implemented"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>D2="Not Assessed"</formula>
-    </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D94" type="list">
-      <formula1>"Implemented,Partial,Not Implemented,Not Assessed"</formula1>
+      <formula1>"Implemented,Partial,Not Implemented"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3849,24 +3867,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3874,54 +3892,54 @@
         <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>